<commit_message>
Day 5 Sprint Implimentation
</commit_message>
<xml_diff>
--- a/IxigoTest/target/test-classes/ExcelData/Data.xlsx
+++ b/IxigoTest/target/test-classes/ExcelData/Data.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Windows.old\Windows\System32\config\systemprofile\eclipse-workspace\My_Project\IxigoTest\src\test\resources\ExcelData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F95FBD1F-6505-4566-A46F-243A63E517DB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B6B9D826-6FF1-44E5-9EAB-87D739B59076}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,12 +25,18 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2" uniqueCount="2">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4" uniqueCount="4">
   <si>
     <t>Goa</t>
   </si>
   <si>
     <t>Destination</t>
+  </si>
+  <si>
+    <t>Area</t>
+  </si>
+  <si>
+    <t>Baga</t>
   </si>
 </sst>
 </file>
@@ -348,20 +354,26 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:A2"/>
+  <dimension ref="A1:B2"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="14.7265625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>1</v>
       </c>
+      <c r="B1" t="s">
+        <v>2</v>
+      </c>
     </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>0</v>
+      </c>
+      <c r="B2" t="s">
+        <v>3</v>
       </c>
     </row>
   </sheetData>

</xml_diff>